<commit_message>
updated to include a assignment having a ? value for a student to represent that it has been submitted to the teacher but not marked yet.  This to show the difference for when something has not been submitted
</commit_message>
<xml_diff>
--- a/Grades.xlsx
+++ b/Grades.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>StudentID</t>
   </si>
@@ -65,6 +65,15 @@
   </si>
   <si>
     <t>Jane</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>DungeonMaster</t>
+  </si>
+  <si>
+    <t>?%</t>
   </si>
   <si>
     <t>Odinson</t>
@@ -90,13 +99,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="2"/>
     </font>
@@ -128,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -153,6 +162,18 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -462,24 +483,24 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="10.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="10" width="39.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="10" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="10" width="18.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="11" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="10.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="14" width="39.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="14" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="14" width="18.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -515,7 +536,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6">
         <v>8701251</v>
       </c>
@@ -551,7 +572,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="6">
         <v>8701252</v>
       </c>
@@ -587,7 +608,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="6">
         <v>8701253</v>
       </c>
@@ -624,38 +645,74 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="6">
+      <c r="A5" s="8">
+        <v>8701255</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="10">
+        <v>0.96</v>
+      </c>
+      <c r="F5" s="10">
+        <v>0.98</v>
+      </c>
+      <c r="G5" s="10">
+        <v>0.94</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0.88</v>
+      </c>
+      <c r="J5" s="10">
+        <v>0.97</v>
+      </c>
+      <c r="K5" s="10">
+        <v>0.93</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+      <c r="A6" s="6">
         <v>8701254</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="7">
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="7">
         <v>0.5</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F6" s="7">
         <v>0</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G6" s="7">
         <v>0.75</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H6" s="7">
         <v>0.86</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I6" s="7">
         <v>0.56</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J6" s="7">
         <v>0.72</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K6" s="7">
         <v>0.87</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L6" s="7">
         <v>0.78</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed report bottom message and updated to use additional column for weighted grade
</commit_message>
<xml_diff>
--- a/Grades.xlsx
+++ b/Grades.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>StudentID</t>
   </si>
@@ -23,6 +23,9 @@
   </si>
   <si>
     <t>First Name</t>
+  </si>
+  <si>
+    <t>Mark</t>
   </si>
   <si>
     <t>1.1 Discussion</t>
@@ -89,7 +92,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +110,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -137,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -157,16 +166,19 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -486,18 +498,18 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="11" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="10.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="14" width="39.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="14" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="14" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="14" width="18.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="13" width="10.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="15" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="15" width="39.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="15" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="15" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="15" width="18.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -510,30 +522,32 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3"/>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E1" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -541,34 +555,36 @@
         <v>8701251</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="7">
+        <v>13</v>
+      </c>
+      <c r="D2" s="7">
+        <v>39</v>
+      </c>
+      <c r="E2" s="8">
         <v>0.67</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="8">
         <v>0.81</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="8">
         <v>0.76</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="8">
         <v>0.58</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="8">
         <v>0.74</v>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="8">
         <v>0.66</v>
       </c>
-      <c r="K2" s="7">
+      <c r="K2" s="8">
         <v>0.88</v>
       </c>
-      <c r="L2" s="7">
+      <c r="L2" s="8">
         <v>0.91</v>
       </c>
     </row>
@@ -577,34 +593,36 @@
         <v>8701252</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="7">
+        <v>15</v>
+      </c>
+      <c r="D3" s="7">
+        <v>98</v>
+      </c>
+      <c r="E3" s="8">
         <v>0.94</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="8">
         <v>0.95</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="8">
         <v>0.89</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="8">
         <v>0.95</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="8">
         <v>0.87</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="8">
         <v>0.76</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="8">
         <v>0.9</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="8">
         <v>0.93</v>
       </c>
     </row>
@@ -613,71 +631,75 @@
         <v>8701253</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="7">
+        <v>17</v>
+      </c>
+      <c r="D4" s="7">
+        <v>7</v>
+      </c>
+      <c r="E4" s="8">
         <v>0.88</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="8">
         <v>0.78</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="8">
         <v>0.79</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="8">
         <v>0.97</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="8">
         <v>0.68</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="8">
         <v>0.85</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="8">
         <v>0.82</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="8">
         <v>0.83</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="8">
+      <c r="A5" s="9">
         <v>8701255</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="10">
+      <c r="C5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="7">
+        <v>99</v>
+      </c>
+      <c r="E5" s="11">
         <v>0.96</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="11">
         <v>0.98</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="11">
         <v>0.94</v>
       </c>
-      <c r="H5" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="10">
+      <c r="H5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="11">
         <v>0.88</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="11">
         <v>0.97</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="11">
         <v>0.93</v>
       </c>
-      <c r="L5" s="10" t="s">
-        <v>19</v>
+      <c r="L5" s="11" t="s">
+        <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
@@ -685,34 +707,36 @@
         <v>8701254</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="7">
+        <v>22</v>
+      </c>
+      <c r="D6" s="7">
+        <v>63</v>
+      </c>
+      <c r="E6" s="8">
         <v>0.5</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="8">
         <v>0</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="8">
         <v>0.75</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="8">
         <v>0.86</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="8">
         <v>0.56</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="8">
         <v>0.72</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="8">
         <v>0.87</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="8">
         <v>0.78</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed centerd grade and wrong date
</commit_message>
<xml_diff>
--- a/Grades.xlsx
+++ b/Grades.xlsx
@@ -146,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -154,8 +154,8 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -166,29 +166,17 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -498,18 +486,18 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="12" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="13" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="13" width="10.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="15" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="15" width="39.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="15" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="15" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="15" width="18.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="10.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="39.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="11" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="11" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="11" width="18.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -637,7 +625,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="7">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="E4" s="8">
         <v>0.88</v>
@@ -664,41 +652,41 @@
         <v>0.83</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="9">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="6">
         <v>8701255</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="7">
         <v>99</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="8">
         <v>0.96</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="8">
         <v>0.98</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="8">
         <v>0.94</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="8">
         <v>0.88</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="8">
         <v>0.97</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="8">
         <v>0.93</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="L5" s="8" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated to use a journal section
</commit_message>
<xml_diff>
--- a/Grades.xlsx
+++ b/Grades.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>StudentID</t>
   </si>
@@ -50,6 +50,15 @@
   </si>
   <si>
     <t>2.22 Food lab Review</t>
+  </si>
+  <si>
+    <t>J1.1</t>
+  </si>
+  <si>
+    <t>J1.2</t>
+  </si>
+  <si>
+    <t>J2.1</t>
   </si>
   <si>
     <t>Smith</t>
@@ -89,10 +98,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,6 +113,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -146,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -154,32 +170,38 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,21 +505,24 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="10.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="10.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="11" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="11" width="39.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="11" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="11" width="18.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="10.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="11" width="10.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="12" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="39.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="12" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="12" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="12" width="18.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -537,42 +562,60 @@
       <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="6">
         <v>8701251</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="7">
+        <v>16</v>
+      </c>
+      <c r="D2" s="6">
         <v>39</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="7">
         <v>0.67</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="7">
         <v>0.81</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="7">
         <v>0.76</v>
       </c>
-      <c r="H2" s="8">
+      <c r="H2" s="7">
         <v>0.58</v>
       </c>
-      <c r="I2" s="8">
+      <c r="I2" s="7">
         <v>0.74</v>
       </c>
-      <c r="J2" s="8">
+      <c r="J2" s="7">
         <v>0.66</v>
       </c>
-      <c r="K2" s="8">
+      <c r="K2" s="7">
         <v>0.88</v>
       </c>
-      <c r="L2" s="8">
+      <c r="L2" s="7">
+        <v>0.91</v>
+      </c>
+      <c r="M2" s="8">
+        <v>0.88</v>
+      </c>
+      <c r="N2" s="8">
+        <v>1</v>
+      </c>
+      <c r="O2" s="7">
         <v>0.91</v>
       </c>
     </row>
@@ -581,36 +624,45 @@
         <v>8701252</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="7">
+        <v>18</v>
+      </c>
+      <c r="D3" s="6">
         <v>98</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="7">
         <v>0.94</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="7">
         <v>0.95</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>0.89</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="7">
         <v>0.95</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="7">
         <v>0.87</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3" s="7">
         <v>0.76</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3" s="7">
         <v>0.9</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="7">
+        <v>0.93</v>
+      </c>
+      <c r="M3" s="8">
+        <v>0.73</v>
+      </c>
+      <c r="N3" s="8">
+        <v>1</v>
+      </c>
+      <c r="O3" s="7">
         <v>0.93</v>
       </c>
     </row>
@@ -619,36 +671,45 @@
         <v>8701253</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="7">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6">
         <v>97</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <v>0.88</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <v>0.78</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>0.79</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>0.97</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="7">
         <v>0.68</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="7">
         <v>0.85</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="7">
         <v>0.82</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="7">
+        <v>0.83</v>
+      </c>
+      <c r="M4" s="8">
+        <v>0.88</v>
+      </c>
+      <c r="N4" s="8">
+        <v>1</v>
+      </c>
+      <c r="O4" s="7">
         <v>0.83</v>
       </c>
     </row>
@@ -657,37 +718,46 @@
         <v>8701255</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="7">
+        <v>22</v>
+      </c>
+      <c r="D5" s="6">
         <v>99</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <v>0.96</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="7">
         <v>0.98</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>0.94</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="8">
+      <c r="H5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="7">
         <v>0.88</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5" s="7">
         <v>0.97</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="7">
         <v>0.93</v>
       </c>
-      <c r="L5" s="8" t="s">
-        <v>20</v>
+      <c r="L5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" s="8">
+        <v>0.97</v>
+      </c>
+      <c r="N5" s="8">
+        <v>1</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>23</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
@@ -695,36 +765,45 @@
         <v>8701254</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="7">
+        <v>25</v>
+      </c>
+      <c r="D6" s="6">
         <v>63</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>0.5</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="7">
         <v>0</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>0.75</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>0.86</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="7">
         <v>0.56</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="7">
         <v>0.72</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="7">
         <v>0.87</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="7">
+        <v>0.78</v>
+      </c>
+      <c r="M6" s="9">
+        <v>0.56</v>
+      </c>
+      <c r="N6" s="8">
+        <v>1</v>
+      </c>
+      <c r="O6" s="7">
         <v>0.78</v>
       </c>
     </row>

</xml_diff>